<commit_message>
Add example row to offline template instructions
</commit_message>
<xml_diff>
--- a/templates/offline_sales_template.xlsx
+++ b/templates/offline_sales_template.xlsx
@@ -35901,7 +35901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -35972,12 +35972,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Do not rename the columns or the sheets. Do not change column D (product_name_auto).</t>
+          <t>Example row: R-2026-0001 | 2026-10-25 | NP-0001 | 1 | (leave empty) | (leave empty)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>Do not rename the columns or the sheets. Do not change column D (product_name_auto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Rows that fail the checks are not loaded. They are listed with a reason in the load report.</t>
         </is>

</xml_diff>